<commit_message>
chore: add tup logo in RSMI pdf
</commit_message>
<xml_diff>
--- a/procurement_documents/RSMI Template.xlsx
+++ b/procurement_documents/RSMI Template.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\emman\itrac\procurement_documents\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{568BBD13-3D83-4108-BB66-735CA555326B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{708857F8-2B11-4DE8-B1DE-C0D13B6FB081}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{E268D2DB-9C06-4916-9525-08CB7B1521D9}"/>
   </bookViews>
@@ -45,6 +45,28 @@
     </ext>
   </extLst>
 </workbook>
+</file>
+
+<file path=xl/metadata.xml><?xml version="1.0" encoding="utf-8"?>
+<metadata xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:xlrd="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata">
+  <metadataTypes count="1">
+    <metadataType name="XLRICHVALUE" minSupportedVersion="120000" copy="1" pasteAll="1" pasteValues="1" merge="1" splitFirst="1" rowColShift="1" clearFormats="1" clearComments="1" assign="1" coerce="1"/>
+  </metadataTypes>
+  <futureMetadata name="XLRICHVALUE" count="1">
+    <bk>
+      <extLst>
+        <ext uri="{3e2802c4-a4d2-4d8b-9148-e3be6c30e623}">
+          <xlrd:rvb i="0"/>
+        </ext>
+      </extLst>
+    </bk>
+  </futureMetadata>
+  <valueMetadata count="1">
+    <bk>
+      <rc t="1" v="0"/>
+    </bk>
+  </valueMetadata>
+</metadata>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
@@ -698,78 +720,7 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="7" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
@@ -798,9 +749,6 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -862,6 +810,87 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="7" fillId="0" borderId="12" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="14" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="13" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="12" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="9" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="10" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="11" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
@@ -873,16 +902,9 @@
     <xf numFmtId="14" fontId="7" fillId="0" borderId="13" xfId="0" quotePrefix="1" applyNumberFormat="1" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -902,80 +924,6 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
-  <xdr:oneCellAnchor>
-    <xdr:from>
-      <xdr:col>0</xdr:col>
-      <xdr:colOff>82826</xdr:colOff>
-      <xdr:row>0</xdr:row>
-      <xdr:rowOff>182218</xdr:rowOff>
-    </xdr:from>
-    <xdr:ext cx="407918" cy="418686"/>
-    <xdr:pic>
-      <xdr:nvPicPr>
-        <xdr:cNvPr id="4" name="Picture 3" descr="C:\Users\arnel olivar\Desktop\logo tup.jpg">
-          <a:extLst>
-            <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{1B68AAC2-BF73-4E70-81E3-DCBBCCEE18DD}"/>
-            </a:ext>
-          </a:extLst>
-        </xdr:cNvPr>
-        <xdr:cNvPicPr>
-          <a:picLocks noChangeAspect="1" noChangeArrowheads="1"/>
-        </xdr:cNvPicPr>
-      </xdr:nvPicPr>
-      <xdr:blipFill>
-        <a:blip xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:embed="rId1">
-          <a:extLst>
-            <a:ext uri="{28A0092B-C50C-407E-A947-70E740481C1C}">
-              <a14:useLocalDpi xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" val="0"/>
-            </a:ext>
-          </a:extLst>
-        </a:blip>
-        <a:srcRect/>
-        <a:stretch>
-          <a:fillRect/>
-        </a:stretch>
-      </xdr:blipFill>
-      <xdr:spPr bwMode="auto">
-        <a:xfrm>
-          <a:off x="82826" y="182218"/>
-          <a:ext cx="407918" cy="418686"/>
-        </a:xfrm>
-        <a:prstGeom prst="rect">
-          <a:avLst/>
-        </a:prstGeom>
-        <a:noFill/>
-        <a:ln>
-          <a:noFill/>
-        </a:ln>
-        <a:extLst>
-          <a:ext uri="{909E8E84-426E-40DD-AFC4-6F175D3DCCD1}">
-            <a14:hiddenFill xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main">
-              <a:solidFill>
-                <a:srgbClr val="FFFFFF"/>
-              </a:solidFill>
-            </a14:hiddenFill>
-          </a:ext>
-          <a:ext uri="{91240B29-F687-4F45-9708-019B960494DF}">
-            <a14:hiddenLine xmlns:a14="http://schemas.microsoft.com/office/drawing/2010/main" w="9525">
-              <a:solidFill>
-                <a:srgbClr val="000000"/>
-              </a:solidFill>
-              <a:miter lim="800000"/>
-              <a:headEnd/>
-              <a:tailEnd/>
-            </a14:hiddenLine>
-          </a:ext>
-        </a:extLst>
-      </xdr:spPr>
-    </xdr:pic>
-    <xdr:clientData/>
-  </xdr:oneCellAnchor>
-</xdr:wsDr>
-</file>
-
-<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:oneCellAnchor>
     <xdr:from>
@@ -1074,6 +1022,70 @@
     </sheetDataSet>
   </externalBook>
 </externalLink>
+</file>
+
+<file path=xl/richData/rdRichValueTypes.xml><?xml version="1.0" encoding="utf-8"?>
+<rvTypesInfo xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" mc:Ignorable="x">
+  <global>
+    <keyFlags>
+      <key name="_Self">
+        <flag name="ExcludeFromFile" value="1"/>
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_DisplayString">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Flags">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Format">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_SubLabel">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Attribution">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Icon">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_Display">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_CanonicalPropertyNames">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+      <key name="_ClassificationId">
+        <flag name="ExcludeFromCalcComparison" value="1"/>
+      </key>
+    </keyFlags>
+  </global>
+</rvTypesInfo>
+</file>
+
+<file path=xl/richData/rdrichvalue.xml><?xml version="1.0" encoding="utf-8"?>
+<rvData xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <rv s="0">
+    <v>0</v>
+    <v>5</v>
+  </rv>
+</rvData>
+</file>
+
+<file path=xl/richData/rdrichvaluestructure.xml><?xml version="1.0" encoding="utf-8"?>
+<rvStructures xmlns="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata" count="1">
+  <s t="_localImage">
+    <k n="_rvRel:LocalImageIdentifier" t="i"/>
+    <k n="CalcOrigin" t="i"/>
+  </s>
+</rvStructures>
+</file>
+
+<file path=xl/richData/richValueRel.xml><?xml version="1.0" encoding="utf-8"?>
+<richValueRels xmlns="http://schemas.microsoft.com/office/spreadsheetml/2022/richvaluerel" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <rel r:id="rId1"/>
+</richValueRels>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1356,127 +1368,129 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="82" t="s">
+      <c r="A1" s="59" t="e" vm="1">
+        <v>#VALUE!</v>
+      </c>
+      <c r="B1" s="60" t="s">
         <v>47</v>
       </c>
-      <c r="B1" s="83"/>
-      <c r="C1" s="83"/>
-      <c r="D1" s="84"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="78"/>
+      <c r="C1" s="60"/>
+      <c r="D1" s="61"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="55"/>
     </row>
     <row r="2" spans="1:9" ht="25.7" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="85"/>
-      <c r="B2" s="86"/>
-      <c r="C2" s="86"/>
-      <c r="D2" s="87"/>
-      <c r="E2" s="79" t="s">
+      <c r="A2" s="62"/>
+      <c r="B2" s="114"/>
+      <c r="C2" s="114"/>
+      <c r="D2" s="63"/>
+      <c r="E2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="81"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="58"/>
     </row>
     <row r="3" spans="1:9" ht="20.85" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="85"/>
-      <c r="B3" s="86"/>
-      <c r="C3" s="86"/>
-      <c r="D3" s="87"/>
-      <c r="E3" s="79" t="s">
+      <c r="A3" s="62"/>
+      <c r="B3" s="114"/>
+      <c r="C3" s="114"/>
+      <c r="D3" s="63"/>
+      <c r="E3" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="81"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="58"/>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="95"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="71"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92" t="s">
+      <c r="A5" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="96" t="s">
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="97"/>
-      <c r="G5" s="97"/>
-      <c r="H5" s="97"/>
-      <c r="I5" s="98"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="74"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="99" t="s">
+      <c r="A6" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="92"/>
-      <c r="C6" s="92"/>
-      <c r="D6" s="99"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="94"/>
-      <c r="G6" s="94"/>
-      <c r="H6" s="94"/>
-      <c r="I6" s="95"/>
+      <c r="B6" s="68"/>
+      <c r="C6" s="68"/>
+      <c r="D6" s="75"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="70"/>
+      <c r="G6" s="70"/>
+      <c r="H6" s="70"/>
+      <c r="I6" s="71"/>
     </row>
     <row r="7" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A7" s="114" t="s">
+      <c r="A7" s="52" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="102"/>
-      <c r="C7" s="102"/>
+      <c r="B7" s="78"/>
+      <c r="C7" s="78"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
-      <c r="F7" s="101" t="s">
+      <c r="F7" s="77" t="s">
         <v>9</v>
       </c>
-      <c r="G7" s="101"/>
-      <c r="H7" s="103"/>
-      <c r="I7" s="104"/>
+      <c r="G7" s="77"/>
+      <c r="H7" s="79"/>
+      <c r="I7" s="80"/>
     </row>
     <row r="8" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="105"/>
-      <c r="C8" s="106"/>
+      <c r="B8" s="81"/>
+      <c r="C8" s="82"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="71" t="s">
+      <c r="F8" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="71"/>
-      <c r="H8" s="72"/>
-      <c r="I8" s="73"/>
+      <c r="G8" s="83"/>
+      <c r="H8" s="84"/>
+      <c r="I8" s="85"/>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="88"/>
-      <c r="B9" s="89"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="89"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="89"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="91" t="s">
+      <c r="A9" s="64"/>
+      <c r="B9" s="65"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="91"/>
+      <c r="I9" s="67"/>
     </row>
     <row r="10" spans="1:9" ht="48.2" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
@@ -1488,10 +1502,10 @@
       <c r="C10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="74" t="s">
+      <c r="D10" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="75"/>
+      <c r="E10" s="87"/>
       <c r="F10" s="6" t="s">
         <v>17</v>
       </c>
@@ -1509,8 +1523,8 @@
       <c r="A11" s="8"/>
       <c r="B11" s="9"/>
       <c r="C11" s="10"/>
-      <c r="D11" s="52"/>
-      <c r="E11" s="53"/>
+      <c r="D11" s="88"/>
+      <c r="E11" s="89"/>
       <c r="F11" s="11"/>
       <c r="G11" s="11"/>
       <c r="H11" s="12"/>
@@ -1520,8 +1534,8 @@
       <c r="A12" s="13"/>
       <c r="B12" s="14"/>
       <c r="C12" s="15"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="53"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="89"/>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
       <c r="H12" s="12"/>
@@ -1531,8 +1545,8 @@
       <c r="A13" s="16"/>
       <c r="B13" s="14"/>
       <c r="C13" s="15"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
+      <c r="D13" s="88"/>
+      <c r="E13" s="89"/>
       <c r="F13" s="11"/>
       <c r="G13" s="17"/>
       <c r="H13" s="12"/>
@@ -1542,8 +1556,8 @@
       <c r="A14" s="18"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="53"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="89"/>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
       <c r="H14" s="12"/>
@@ -1553,8 +1567,8 @@
       <c r="A15" s="19"/>
       <c r="B15" s="20"/>
       <c r="C15" s="15"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="53"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="89"/>
       <c r="F15" s="11"/>
       <c r="G15" s="21"/>
       <c r="H15" s="12"/>
@@ -1564,8 +1578,8 @@
       <c r="A16" s="18"/>
       <c r="B16" s="20"/>
       <c r="C16" s="15"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="53"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="89"/>
       <c r="F16" s="11"/>
       <c r="G16" s="21"/>
       <c r="H16" s="12"/>
@@ -1575,8 +1589,8 @@
       <c r="A17" s="22"/>
       <c r="B17" s="14"/>
       <c r="C17" s="15"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="89"/>
       <c r="F17" s="11"/>
       <c r="G17" s="21"/>
       <c r="H17" s="12"/>
@@ -1589,8 +1603,8 @@
       <c r="A18" s="18"/>
       <c r="B18" s="14"/>
       <c r="C18" s="15"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="53"/>
+      <c r="D18" s="88"/>
+      <c r="E18" s="89"/>
       <c r="F18" s="11"/>
       <c r="G18" s="21"/>
       <c r="H18" s="12"/>
@@ -1600,8 +1614,8 @@
       <c r="A19" s="19"/>
       <c r="B19" s="23"/>
       <c r="C19" s="15"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="89"/>
       <c r="F19" s="11"/>
       <c r="G19" s="24"/>
       <c r="H19" s="12"/>
@@ -1611,8 +1625,8 @@
       <c r="A20" s="18"/>
       <c r="B20" s="14"/>
       <c r="C20" s="15"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="89"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
       <c r="H20" s="12"/>
@@ -1625,8 +1639,8 @@
       <c r="A21" s="18"/>
       <c r="B21" s="14"/>
       <c r="C21" s="15"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="89"/>
       <c r="F21" s="11"/>
       <c r="G21" s="11"/>
       <c r="H21" s="12"/>
@@ -1636,8 +1650,8 @@
       <c r="A22" s="18"/>
       <c r="B22" s="14"/>
       <c r="C22" s="15"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="53"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="89"/>
       <c r="F22" s="11"/>
       <c r="G22" s="25"/>
       <c r="H22" s="12"/>
@@ -1647,8 +1661,8 @@
       <c r="A23" s="18"/>
       <c r="B23" s="14"/>
       <c r="C23" s="15"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="53"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="89"/>
       <c r="F23" s="11"/>
       <c r="G23" s="26"/>
       <c r="H23" s="12"/>
@@ -1658,8 +1672,8 @@
       <c r="A24" s="18"/>
       <c r="B24" s="14"/>
       <c r="C24" s="15"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="53"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="89"/>
       <c r="F24" s="11"/>
       <c r="G24" s="26"/>
       <c r="H24" s="12"/>
@@ -1672,8 +1686,8 @@
       <c r="A25" s="18"/>
       <c r="B25" s="14"/>
       <c r="C25" s="15"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53"/>
+      <c r="D25" s="88"/>
+      <c r="E25" s="89"/>
       <c r="F25" s="11"/>
       <c r="G25" s="26"/>
       <c r="H25" s="12"/>
@@ -1683,8 +1697,8 @@
       <c r="A26" s="18"/>
       <c r="B26" s="14"/>
       <c r="C26" s="15"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="53"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="89"/>
       <c r="F26" s="11"/>
       <c r="G26" s="26"/>
       <c r="H26" s="12"/>
@@ -1694,8 +1708,8 @@
       <c r="A27" s="18"/>
       <c r="B27" s="14"/>
       <c r="C27" s="15"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
+      <c r="D27" s="88"/>
+      <c r="E27" s="89"/>
       <c r="F27" s="11"/>
       <c r="G27" s="26"/>
       <c r="H27" s="12"/>
@@ -1705,8 +1719,8 @@
       <c r="A28" s="18"/>
       <c r="B28" s="14"/>
       <c r="C28" s="15"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="53"/>
+      <c r="D28" s="88"/>
+      <c r="E28" s="89"/>
       <c r="F28" s="11"/>
       <c r="G28" s="26"/>
       <c r="H28" s="12"/>
@@ -1716,8 +1730,8 @@
       <c r="A29" s="18"/>
       <c r="B29" s="14"/>
       <c r="C29" s="15"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="53"/>
+      <c r="D29" s="88"/>
+      <c r="E29" s="89"/>
       <c r="F29" s="11"/>
       <c r="G29" s="26"/>
       <c r="H29" s="12"/>
@@ -1727,8 +1741,8 @@
       <c r="A30" s="18"/>
       <c r="B30" s="14"/>
       <c r="C30" s="15"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="53"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="89"/>
       <c r="F30" s="11"/>
       <c r="G30" s="26"/>
       <c r="H30" s="12"/>
@@ -1738,8 +1752,8 @@
       <c r="A31" s="18"/>
       <c r="B31" s="14"/>
       <c r="C31" s="15"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="89"/>
       <c r="F31" s="11"/>
       <c r="G31" s="26"/>
       <c r="H31" s="12"/>
@@ -1749,8 +1763,8 @@
       <c r="A32" s="18"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="53"/>
+      <c r="D32" s="88"/>
+      <c r="E32" s="89"/>
       <c r="F32" s="11"/>
       <c r="G32" s="21"/>
       <c r="H32" s="12"/>
@@ -1760,8 +1774,8 @@
       <c r="A33" s="18"/>
       <c r="B33" s="14"/>
       <c r="C33" s="15"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="53"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="89"/>
       <c r="F33" s="27"/>
       <c r="G33" s="21"/>
       <c r="H33" s="12"/>
@@ -1771,8 +1785,8 @@
       <c r="A34" s="18"/>
       <c r="B34" s="14"/>
       <c r="C34" s="15"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="53"/>
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
       <c r="F34" s="11"/>
       <c r="G34" s="21"/>
       <c r="H34" s="12"/>
@@ -1782,8 +1796,8 @@
       <c r="A35" s="18"/>
       <c r="B35" s="14"/>
       <c r="C35" s="15"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
+      <c r="D35" s="88"/>
+      <c r="E35" s="89"/>
       <c r="F35" s="11"/>
       <c r="G35" s="21"/>
       <c r="H35" s="12"/>
@@ -1793,8 +1807,8 @@
       <c r="A36" s="18"/>
       <c r="B36" s="14"/>
       <c r="C36" s="15"/>
-      <c r="D36" s="52"/>
-      <c r="E36" s="53"/>
+      <c r="D36" s="88"/>
+      <c r="E36" s="89"/>
       <c r="F36" s="11"/>
       <c r="G36" s="21"/>
       <c r="H36" s="12"/>
@@ -1804,8 +1818,8 @@
       <c r="A37" s="18"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="53"/>
+      <c r="D37" s="88"/>
+      <c r="E37" s="89"/>
       <c r="F37" s="11"/>
       <c r="G37" s="21"/>
       <c r="H37" s="12"/>
@@ -1815,8 +1829,8 @@
       <c r="A38" s="18"/>
       <c r="B38" s="14"/>
       <c r="C38" s="15"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="53"/>
+      <c r="D38" s="88"/>
+      <c r="E38" s="89"/>
       <c r="F38" s="11"/>
       <c r="G38" s="21"/>
       <c r="H38" s="12"/>
@@ -1826,8 +1840,8 @@
       <c r="A39" s="18"/>
       <c r="B39" s="14"/>
       <c r="C39" s="15"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="53"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="89"/>
       <c r="F39" s="11"/>
       <c r="G39" s="21"/>
       <c r="H39" s="12"/>
@@ -1837,8 +1851,8 @@
       <c r="A40" s="18"/>
       <c r="B40" s="14"/>
       <c r="C40" s="15"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="53"/>
+      <c r="D40" s="88"/>
+      <c r="E40" s="89"/>
       <c r="F40" s="28"/>
       <c r="G40" s="29"/>
       <c r="H40" s="12"/>
@@ -1848,32 +1862,32 @@
       <c r="A41" s="18"/>
       <c r="B41" s="31"/>
       <c r="C41" s="15"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="65" t="s">
+      <c r="D41" s="88"/>
+      <c r="E41" s="89"/>
+      <c r="F41" s="90" t="s">
         <v>23</v>
       </c>
-      <c r="G41" s="66"/>
-      <c r="H41" s="67"/>
+      <c r="G41" s="91"/>
+      <c r="H41" s="92"/>
       <c r="I41" s="12">
         <f>SUM(I11:I40)</f>
         <v>0</v>
       </c>
     </row>
     <row r="42" spans="1:13" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A42" s="68" t="s">
+      <c r="A42" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="69"/>
+      <c r="B42" s="94"/>
       <c r="C42" s="34"/>
       <c r="D42" s="35"/>
       <c r="E42" s="36"/>
       <c r="F42" s="36"/>
-      <c r="G42" s="68" t="s">
+      <c r="G42" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="H42" s="70"/>
-      <c r="I42" s="69"/>
+      <c r="H42" s="95"/>
+      <c r="I42" s="94"/>
     </row>
     <row r="43" spans="1:13" ht="35.85" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="37" t="s">
@@ -1954,69 +1968,69 @@
       <c r="I48" s="50"/>
     </row>
     <row r="49" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A49" s="54"/>
-      <c r="B49" s="55"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="56"/>
+      <c r="A49" s="96"/>
+      <c r="B49" s="97"/>
+      <c r="C49" s="97"/>
+      <c r="D49" s="97"/>
+      <c r="E49" s="98"/>
+      <c r="F49" s="96"/>
+      <c r="G49" s="97"/>
+      <c r="H49" s="97"/>
+      <c r="I49" s="98"/>
     </row>
     <row r="50" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A50" s="54"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="56"/>
-      <c r="F50" s="54"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
+      <c r="A50" s="96"/>
+      <c r="B50" s="97"/>
+      <c r="C50" s="97"/>
+      <c r="D50" s="97"/>
+      <c r="E50" s="98"/>
+      <c r="F50" s="96"/>
+      <c r="G50" s="97"/>
+      <c r="H50" s="97"/>
+      <c r="I50" s="98"/>
     </row>
     <row r="51" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A51" s="60"/>
-      <c r="B51" s="61"/>
-      <c r="C51" s="61"/>
-      <c r="D51" s="61"/>
-      <c r="E51" s="62"/>
-      <c r="F51" s="63" t="s">
+      <c r="A51" s="102"/>
+      <c r="B51" s="103"/>
+      <c r="C51" s="103"/>
+      <c r="D51" s="103"/>
+      <c r="E51" s="104"/>
+      <c r="F51" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="G51" s="64"/>
-      <c r="H51" s="64"/>
+      <c r="G51" s="106"/>
+      <c r="H51" s="106"/>
       <c r="I51" s="51" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:9" ht="15.95" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="54" t="s">
+      <c r="A52" s="96" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="55"/>
-      <c r="C52" s="55"/>
-      <c r="D52" s="55"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="54" t="s">
+      <c r="B52" s="97"/>
+      <c r="C52" s="97"/>
+      <c r="D52" s="97"/>
+      <c r="E52" s="98"/>
+      <c r="F52" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="G52" s="55"/>
-      <c r="H52" s="55"/>
+      <c r="G52" s="97"/>
+      <c r="H52" s="97"/>
       <c r="I52" s="51" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A53" s="57"/>
-      <c r="B53" s="58"/>
-      <c r="C53" s="58"/>
-      <c r="D53" s="58"/>
-      <c r="E53" s="59"/>
-      <c r="F53" s="57"/>
-      <c r="G53" s="58"/>
-      <c r="H53" s="58"/>
-      <c r="I53" s="59"/>
+      <c r="A53" s="99"/>
+      <c r="B53" s="100"/>
+      <c r="C53" s="100"/>
+      <c r="D53" s="100"/>
+      <c r="E53" s="101"/>
+      <c r="F53" s="99"/>
+      <c r="G53" s="100"/>
+      <c r="H53" s="100"/>
+      <c r="I53" s="101"/>
     </row>
     <row r="54" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2084,29 +2098,34 @@
     <row r="163" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="166" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
-  <mergeCells count="63">
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="E3:I3"/>
-    <mergeCell ref="A1:D3"/>
-    <mergeCell ref="A9:G9"/>
-    <mergeCell ref="H9:I9"/>
-    <mergeCell ref="A4:D4"/>
-    <mergeCell ref="E4:I4"/>
-    <mergeCell ref="A5:D5"/>
-    <mergeCell ref="E5:I5"/>
-    <mergeCell ref="A6:D6"/>
-    <mergeCell ref="E6:I6"/>
-    <mergeCell ref="F7:G7"/>
-    <mergeCell ref="B7:C7"/>
-    <mergeCell ref="H7:I7"/>
-    <mergeCell ref="B8:C8"/>
-    <mergeCell ref="F8:G8"/>
-    <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D30:E30"/>
+  <mergeCells count="64">
+    <mergeCell ref="B1:D3"/>
+    <mergeCell ref="A1:A3"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="D33:E33"/>
     <mergeCell ref="F41:H41"/>
     <mergeCell ref="A42:B42"/>
     <mergeCell ref="G42:I42"/>
@@ -2123,35 +2142,30 @@
     <mergeCell ref="D27:E27"/>
     <mergeCell ref="D28:E28"/>
     <mergeCell ref="D29:E29"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="F52:H52"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="F8:G8"/>
+    <mergeCell ref="H8:I8"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="A9:G9"/>
+    <mergeCell ref="H9:I9"/>
+    <mergeCell ref="A4:D4"/>
+    <mergeCell ref="E4:I4"/>
+    <mergeCell ref="A5:D5"/>
+    <mergeCell ref="E5:I5"/>
+    <mergeCell ref="A6:D6"/>
+    <mergeCell ref="E6:I6"/>
+    <mergeCell ref="F7:G7"/>
+    <mergeCell ref="B7:C7"/>
+    <mergeCell ref="H7:I7"/>
+    <mergeCell ref="B8:C8"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.47244094488188981" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" r:id="rId1"/>
-  <drawing r:id="rId2"/>
 </worksheet>
 </file>
 
@@ -2174,137 +2188,137 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="111" t="s">
+      <c r="A1" s="107" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="111"/>
-      <c r="C1" s="111"/>
-      <c r="D1" s="111"/>
-      <c r="E1" s="76"/>
-      <c r="F1" s="77"/>
-      <c r="G1" s="77"/>
-      <c r="H1" s="77"/>
-      <c r="I1" s="78"/>
+      <c r="B1" s="107"/>
+      <c r="C1" s="107"/>
+      <c r="D1" s="107"/>
+      <c r="E1" s="53"/>
+      <c r="F1" s="54"/>
+      <c r="G1" s="54"/>
+      <c r="H1" s="54"/>
+      <c r="I1" s="55"/>
     </row>
     <row r="2" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A2" s="112" t="s">
+      <c r="A2" s="108" t="s">
         <v>1</v>
       </c>
-      <c r="B2" s="112"/>
-      <c r="C2" s="112"/>
-      <c r="D2" s="112"/>
-      <c r="E2" s="79" t="s">
+      <c r="B2" s="108"/>
+      <c r="C2" s="108"/>
+      <c r="D2" s="108"/>
+      <c r="E2" s="56" t="s">
         <v>2</v>
       </c>
-      <c r="F2" s="80"/>
-      <c r="G2" s="80"/>
-      <c r="H2" s="80"/>
-      <c r="I2" s="81"/>
+      <c r="F2" s="57"/>
+      <c r="G2" s="57"/>
+      <c r="H2" s="57"/>
+      <c r="I2" s="58"/>
     </row>
     <row r="3" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="113"/>
-      <c r="B3" s="113"/>
-      <c r="C3" s="113"/>
-      <c r="D3" s="113"/>
-      <c r="E3" s="79" t="s">
+      <c r="A3" s="109"/>
+      <c r="B3" s="109"/>
+      <c r="C3" s="109"/>
+      <c r="D3" s="109"/>
+      <c r="E3" s="56" t="s">
         <v>3</v>
       </c>
-      <c r="F3" s="80"/>
-      <c r="G3" s="80"/>
-      <c r="H3" s="80"/>
-      <c r="I3" s="81"/>
+      <c r="F3" s="57"/>
+      <c r="G3" s="57"/>
+      <c r="H3" s="57"/>
+      <c r="I3" s="58"/>
     </row>
     <row r="4" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A4" s="92" t="s">
+      <c r="A4" s="68" t="s">
         <v>4</v>
       </c>
-      <c r="B4" s="92"/>
-      <c r="C4" s="92"/>
-      <c r="D4" s="92"/>
-      <c r="E4" s="93"/>
-      <c r="F4" s="94"/>
-      <c r="G4" s="94"/>
-      <c r="H4" s="94"/>
-      <c r="I4" s="95"/>
+      <c r="B4" s="68"/>
+      <c r="C4" s="68"/>
+      <c r="D4" s="68"/>
+      <c r="E4" s="69"/>
+      <c r="F4" s="70"/>
+      <c r="G4" s="70"/>
+      <c r="H4" s="70"/>
+      <c r="I4" s="71"/>
     </row>
     <row r="5" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A5" s="92" t="s">
+      <c r="A5" s="68" t="s">
         <v>5</v>
       </c>
-      <c r="B5" s="92"/>
-      <c r="C5" s="92"/>
-      <c r="D5" s="92"/>
-      <c r="E5" s="96" t="s">
+      <c r="B5" s="68"/>
+      <c r="C5" s="68"/>
+      <c r="D5" s="68"/>
+      <c r="E5" s="72" t="s">
         <v>6</v>
       </c>
-      <c r="F5" s="97"/>
-      <c r="G5" s="97"/>
-      <c r="H5" s="97"/>
-      <c r="I5" s="98"/>
+      <c r="F5" s="73"/>
+      <c r="G5" s="73"/>
+      <c r="H5" s="73"/>
+      <c r="I5" s="74"/>
     </row>
     <row r="6" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A6" s="99" t="s">
+      <c r="A6" s="75" t="s">
         <v>7</v>
       </c>
-      <c r="B6" s="99"/>
-      <c r="C6" s="99"/>
-      <c r="D6" s="99"/>
-      <c r="E6" s="100"/>
-      <c r="F6" s="107"/>
-      <c r="G6" s="107"/>
-      <c r="H6" s="107"/>
-      <c r="I6" s="108"/>
+      <c r="B6" s="75"/>
+      <c r="C6" s="75"/>
+      <c r="D6" s="75"/>
+      <c r="E6" s="76"/>
+      <c r="F6" s="110"/>
+      <c r="G6" s="110"/>
+      <c r="H6" s="110"/>
+      <c r="I6" s="111"/>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="B7" s="109" t="s">
+      <c r="B7" s="112" t="s">
         <v>33</v>
       </c>
-      <c r="C7" s="109"/>
+      <c r="C7" s="112"/>
       <c r="D7" s="2"/>
       <c r="E7" s="3"/>
       <c r="F7" s="2" t="s">
         <v>9</v>
       </c>
       <c r="G7" s="2"/>
-      <c r="H7" s="103" t="s">
+      <c r="H7" s="79" t="s">
         <v>35</v>
       </c>
-      <c r="I7" s="110"/>
+      <c r="I7" s="113"/>
     </row>
     <row r="8" spans="1:9" x14ac:dyDescent="0.25">
       <c r="A8" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B8" s="105" t="s">
+      <c r="B8" s="81" t="s">
         <v>34</v>
       </c>
-      <c r="C8" s="106"/>
+      <c r="C8" s="82"/>
       <c r="D8" s="2"/>
       <c r="E8" s="2"/>
-      <c r="F8" s="71" t="s">
+      <c r="F8" s="83" t="s">
         <v>11</v>
       </c>
-      <c r="G8" s="71"/>
-      <c r="H8" s="72" t="s">
+      <c r="G8" s="83"/>
+      <c r="H8" s="84" t="s">
         <v>36</v>
       </c>
-      <c r="I8" s="73"/>
+      <c r="I8" s="85"/>
     </row>
     <row r="9" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A9" s="88"/>
-      <c r="B9" s="89"/>
-      <c r="C9" s="89"/>
-      <c r="D9" s="89"/>
-      <c r="E9" s="89"/>
-      <c r="F9" s="89"/>
-      <c r="G9" s="90"/>
-      <c r="H9" s="91" t="s">
+      <c r="A9" s="64"/>
+      <c r="B9" s="65"/>
+      <c r="C9" s="65"/>
+      <c r="D9" s="65"/>
+      <c r="E9" s="65"/>
+      <c r="F9" s="65"/>
+      <c r="G9" s="66"/>
+      <c r="H9" s="67" t="s">
         <v>12</v>
       </c>
-      <c r="I9" s="91"/>
+      <c r="I9" s="67"/>
     </row>
     <row r="10" spans="1:9" ht="33.75" x14ac:dyDescent="0.25">
       <c r="A10" s="6" t="s">
@@ -2316,10 +2330,10 @@
       <c r="C10" s="6" t="s">
         <v>15</v>
       </c>
-      <c r="D10" s="74" t="s">
+      <c r="D10" s="86" t="s">
         <v>16</v>
       </c>
-      <c r="E10" s="75"/>
+      <c r="E10" s="87"/>
       <c r="F10" s="6" t="s">
         <v>17</v>
       </c>
@@ -2343,10 +2357,10 @@
       <c r="C11" s="10" t="s">
         <v>41</v>
       </c>
-      <c r="D11" s="52" t="s">
+      <c r="D11" s="88" t="s">
         <v>42</v>
       </c>
-      <c r="E11" s="53"/>
+      <c r="E11" s="89"/>
       <c r="F11" s="11" t="s">
         <v>43</v>
       </c>
@@ -2364,8 +2378,8 @@
       <c r="A12" s="13"/>
       <c r="B12" s="14"/>
       <c r="C12" s="15"/>
-      <c r="D12" s="52"/>
-      <c r="E12" s="53"/>
+      <c r="D12" s="88"/>
+      <c r="E12" s="89"/>
       <c r="F12" s="11"/>
       <c r="G12" s="11"/>
       <c r="H12" s="12"/>
@@ -2375,8 +2389,8 @@
       <c r="A13" s="16"/>
       <c r="B13" s="14"/>
       <c r="C13" s="15"/>
-      <c r="D13" s="52"/>
-      <c r="E13" s="53"/>
+      <c r="D13" s="88"/>
+      <c r="E13" s="89"/>
       <c r="F13" s="11"/>
       <c r="G13" s="17"/>
       <c r="H13" s="12"/>
@@ -2386,8 +2400,8 @@
       <c r="A14" s="18"/>
       <c r="B14" s="14"/>
       <c r="C14" s="15"/>
-      <c r="D14" s="52"/>
-      <c r="E14" s="53"/>
+      <c r="D14" s="88"/>
+      <c r="E14" s="89"/>
       <c r="F14" s="11"/>
       <c r="G14" s="11"/>
       <c r="H14" s="12"/>
@@ -2397,8 +2411,8 @@
       <c r="A15" s="19"/>
       <c r="B15" s="20"/>
       <c r="C15" s="15"/>
-      <c r="D15" s="52"/>
-      <c r="E15" s="53"/>
+      <c r="D15" s="88"/>
+      <c r="E15" s="89"/>
       <c r="F15" s="11"/>
       <c r="G15" s="21"/>
       <c r="H15" s="12"/>
@@ -2408,8 +2422,8 @@
       <c r="A16" s="18"/>
       <c r="B16" s="20"/>
       <c r="C16" s="15"/>
-      <c r="D16" s="52"/>
-      <c r="E16" s="53"/>
+      <c r="D16" s="88"/>
+      <c r="E16" s="89"/>
       <c r="F16" s="11"/>
       <c r="G16" s="21"/>
       <c r="H16" s="12"/>
@@ -2419,8 +2433,8 @@
       <c r="A17" s="22"/>
       <c r="B17" s="14"/>
       <c r="C17" s="15"/>
-      <c r="D17" s="52"/>
-      <c r="E17" s="53"/>
+      <c r="D17" s="88"/>
+      <c r="E17" s="89"/>
       <c r="F17" s="11"/>
       <c r="G17" s="21"/>
       <c r="H17" s="12"/>
@@ -2433,8 +2447,8 @@
       <c r="A18" s="18"/>
       <c r="B18" s="14"/>
       <c r="C18" s="15"/>
-      <c r="D18" s="52"/>
-      <c r="E18" s="53"/>
+      <c r="D18" s="88"/>
+      <c r="E18" s="89"/>
       <c r="F18" s="11"/>
       <c r="G18" s="21"/>
       <c r="H18" s="12"/>
@@ -2444,8 +2458,8 @@
       <c r="A19" s="19"/>
       <c r="B19" s="23"/>
       <c r="C19" s="15"/>
-      <c r="D19" s="52"/>
-      <c r="E19" s="53"/>
+      <c r="D19" s="88"/>
+      <c r="E19" s="89"/>
       <c r="F19" s="11"/>
       <c r="G19" s="24"/>
       <c r="H19" s="12"/>
@@ -2455,8 +2469,8 @@
       <c r="A20" s="18"/>
       <c r="B20" s="14"/>
       <c r="C20" s="15"/>
-      <c r="D20" s="52"/>
-      <c r="E20" s="53"/>
+      <c r="D20" s="88"/>
+      <c r="E20" s="89"/>
       <c r="F20" s="11"/>
       <c r="G20" s="11"/>
       <c r="H20" s="12"/>
@@ -2469,8 +2483,8 @@
       <c r="A21" s="18"/>
       <c r="B21" s="14"/>
       <c r="C21" s="15"/>
-      <c r="D21" s="52"/>
-      <c r="E21" s="53"/>
+      <c r="D21" s="88"/>
+      <c r="E21" s="89"/>
       <c r="F21" s="11"/>
       <c r="G21" s="11"/>
       <c r="H21" s="12"/>
@@ -2480,8 +2494,8 @@
       <c r="A22" s="18"/>
       <c r="B22" s="14"/>
       <c r="C22" s="15"/>
-      <c r="D22" s="52"/>
-      <c r="E22" s="53"/>
+      <c r="D22" s="88"/>
+      <c r="E22" s="89"/>
       <c r="F22" s="11"/>
       <c r="G22" s="25"/>
       <c r="H22" s="12"/>
@@ -2491,8 +2505,8 @@
       <c r="A23" s="18"/>
       <c r="B23" s="14"/>
       <c r="C23" s="15"/>
-      <c r="D23" s="52"/>
-      <c r="E23" s="53"/>
+      <c r="D23" s="88"/>
+      <c r="E23" s="89"/>
       <c r="F23" s="11"/>
       <c r="G23" s="26"/>
       <c r="H23" s="12"/>
@@ -2502,8 +2516,8 @@
       <c r="A24" s="18"/>
       <c r="B24" s="14"/>
       <c r="C24" s="15"/>
-      <c r="D24" s="52"/>
-      <c r="E24" s="53"/>
+      <c r="D24" s="88"/>
+      <c r="E24" s="89"/>
       <c r="F24" s="11"/>
       <c r="G24" s="26"/>
       <c r="H24" s="12"/>
@@ -2516,8 +2530,8 @@
       <c r="A25" s="18"/>
       <c r="B25" s="14"/>
       <c r="C25" s="15"/>
-      <c r="D25" s="52"/>
-      <c r="E25" s="53"/>
+      <c r="D25" s="88"/>
+      <c r="E25" s="89"/>
       <c r="F25" s="11"/>
       <c r="G25" s="26"/>
       <c r="H25" s="12"/>
@@ -2527,8 +2541,8 @@
       <c r="A26" s="18"/>
       <c r="B26" s="14"/>
       <c r="C26" s="15"/>
-      <c r="D26" s="52"/>
-      <c r="E26" s="53"/>
+      <c r="D26" s="88"/>
+      <c r="E26" s="89"/>
       <c r="F26" s="11"/>
       <c r="G26" s="26"/>
       <c r="H26" s="12"/>
@@ -2538,8 +2552,8 @@
       <c r="A27" s="18"/>
       <c r="B27" s="14"/>
       <c r="C27" s="15"/>
-      <c r="D27" s="52"/>
-      <c r="E27" s="53"/>
+      <c r="D27" s="88"/>
+      <c r="E27" s="89"/>
       <c r="F27" s="11"/>
       <c r="G27" s="26"/>
       <c r="H27" s="12"/>
@@ -2549,8 +2563,8 @@
       <c r="A28" s="18"/>
       <c r="B28" s="14"/>
       <c r="C28" s="15"/>
-      <c r="D28" s="52"/>
-      <c r="E28" s="53"/>
+      <c r="D28" s="88"/>
+      <c r="E28" s="89"/>
       <c r="F28" s="11"/>
       <c r="G28" s="26"/>
       <c r="H28" s="12"/>
@@ -2560,8 +2574,8 @@
       <c r="A29" s="18"/>
       <c r="B29" s="14"/>
       <c r="C29" s="15"/>
-      <c r="D29" s="52"/>
-      <c r="E29" s="53"/>
+      <c r="D29" s="88"/>
+      <c r="E29" s="89"/>
       <c r="F29" s="11"/>
       <c r="G29" s="26"/>
       <c r="H29" s="12"/>
@@ -2571,8 +2585,8 @@
       <c r="A30" s="18"/>
       <c r="B30" s="14"/>
       <c r="C30" s="15"/>
-      <c r="D30" s="52"/>
-      <c r="E30" s="53"/>
+      <c r="D30" s="88"/>
+      <c r="E30" s="89"/>
       <c r="F30" s="11"/>
       <c r="G30" s="26"/>
       <c r="H30" s="12"/>
@@ -2582,8 +2596,8 @@
       <c r="A31" s="18"/>
       <c r="B31" s="14"/>
       <c r="C31" s="15"/>
-      <c r="D31" s="52"/>
-      <c r="E31" s="53"/>
+      <c r="D31" s="88"/>
+      <c r="E31" s="89"/>
       <c r="F31" s="11"/>
       <c r="G31" s="26"/>
       <c r="H31" s="12"/>
@@ -2593,8 +2607,8 @@
       <c r="A32" s="18"/>
       <c r="B32" s="14"/>
       <c r="C32" s="15"/>
-      <c r="D32" s="52"/>
-      <c r="E32" s="53"/>
+      <c r="D32" s="88"/>
+      <c r="E32" s="89"/>
       <c r="F32" s="11"/>
       <c r="G32" s="21"/>
       <c r="H32" s="12"/>
@@ -2604,8 +2618,8 @@
       <c r="A33" s="18"/>
       <c r="B33" s="14"/>
       <c r="C33" s="15"/>
-      <c r="D33" s="52"/>
-      <c r="E33" s="53"/>
+      <c r="D33" s="88"/>
+      <c r="E33" s="89"/>
       <c r="F33" s="27"/>
       <c r="G33" s="21"/>
       <c r="H33" s="12"/>
@@ -2615,8 +2629,8 @@
       <c r="A34" s="18"/>
       <c r="B34" s="14"/>
       <c r="C34" s="15"/>
-      <c r="D34" s="52"/>
-      <c r="E34" s="53"/>
+      <c r="D34" s="88"/>
+      <c r="E34" s="89"/>
       <c r="F34" s="11"/>
       <c r="G34" s="21"/>
       <c r="H34" s="12"/>
@@ -2626,8 +2640,8 @@
       <c r="A35" s="18"/>
       <c r="B35" s="14"/>
       <c r="C35" s="15"/>
-      <c r="D35" s="52"/>
-      <c r="E35" s="53"/>
+      <c r="D35" s="88"/>
+      <c r="E35" s="89"/>
       <c r="F35" s="11"/>
       <c r="G35" s="21"/>
       <c r="H35" s="12"/>
@@ -2637,8 +2651,8 @@
       <c r="A36" s="18"/>
       <c r="B36" s="14"/>
       <c r="C36" s="15"/>
-      <c r="D36" s="52"/>
-      <c r="E36" s="53"/>
+      <c r="D36" s="88"/>
+      <c r="E36" s="89"/>
       <c r="F36" s="11"/>
       <c r="G36" s="21"/>
       <c r="H36" s="12"/>
@@ -2648,8 +2662,8 @@
       <c r="A37" s="18"/>
       <c r="B37" s="14"/>
       <c r="C37" s="15"/>
-      <c r="D37" s="52"/>
-      <c r="E37" s="53"/>
+      <c r="D37" s="88"/>
+      <c r="E37" s="89"/>
       <c r="F37" s="11"/>
       <c r="G37" s="21"/>
       <c r="H37" s="12"/>
@@ -2659,8 +2673,8 @@
       <c r="A38" s="18"/>
       <c r="B38" s="14"/>
       <c r="C38" s="15"/>
-      <c r="D38" s="52"/>
-      <c r="E38" s="53"/>
+      <c r="D38" s="88"/>
+      <c r="E38" s="89"/>
       <c r="F38" s="11"/>
       <c r="G38" s="21"/>
       <c r="H38" s="12"/>
@@ -2670,8 +2684,8 @@
       <c r="A39" s="18"/>
       <c r="B39" s="14"/>
       <c r="C39" s="15"/>
-      <c r="D39" s="52"/>
-      <c r="E39" s="53"/>
+      <c r="D39" s="88"/>
+      <c r="E39" s="89"/>
       <c r="F39" s="11"/>
       <c r="G39" s="21"/>
       <c r="H39" s="12"/>
@@ -2681,8 +2695,8 @@
       <c r="A40" s="18"/>
       <c r="B40" s="14"/>
       <c r="C40" s="15"/>
-      <c r="D40" s="52"/>
-      <c r="E40" s="53"/>
+      <c r="D40" s="88"/>
+      <c r="E40" s="89"/>
       <c r="F40" s="28"/>
       <c r="G40" s="29"/>
       <c r="H40" s="12"/>
@@ -2692,31 +2706,31 @@
       <c r="A41" s="18"/>
       <c r="B41" s="31"/>
       <c r="C41" s="15"/>
-      <c r="D41" s="52"/>
-      <c r="E41" s="53"/>
-      <c r="F41" s="65" t="s">
+      <c r="D41" s="88"/>
+      <c r="E41" s="89"/>
+      <c r="F41" s="90" t="s">
         <v>23</v>
       </c>
-      <c r="G41" s="66"/>
-      <c r="H41" s="67"/>
+      <c r="G41" s="91"/>
+      <c r="H41" s="92"/>
       <c r="I41" s="12" t="s">
         <v>37</v>
       </c>
     </row>
     <row r="42" spans="1:13" x14ac:dyDescent="0.25">
-      <c r="A42" s="68" t="s">
+      <c r="A42" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="B42" s="69"/>
+      <c r="B42" s="94"/>
       <c r="C42" s="34"/>
       <c r="D42" s="35"/>
       <c r="E42" s="36"/>
       <c r="F42" s="36"/>
-      <c r="G42" s="68" t="s">
+      <c r="G42" s="93" t="s">
         <v>24</v>
       </c>
-      <c r="H42" s="70"/>
-      <c r="I42" s="69"/>
+      <c r="H42" s="95"/>
+      <c r="I42" s="94"/>
     </row>
     <row r="43" spans="1:13" ht="22.5" x14ac:dyDescent="0.25">
       <c r="A43" s="37" t="s">
@@ -2797,71 +2811,71 @@
       <c r="I48" s="50"/>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A49" s="54"/>
-      <c r="B49" s="55"/>
-      <c r="C49" s="55"/>
-      <c r="D49" s="55"/>
-      <c r="E49" s="56"/>
-      <c r="F49" s="54"/>
-      <c r="G49" s="55"/>
-      <c r="H49" s="55"/>
-      <c r="I49" s="56"/>
+      <c r="A49" s="96"/>
+      <c r="B49" s="97"/>
+      <c r="C49" s="97"/>
+      <c r="D49" s="97"/>
+      <c r="E49" s="98"/>
+      <c r="F49" s="96"/>
+      <c r="G49" s="97"/>
+      <c r="H49" s="97"/>
+      <c r="I49" s="98"/>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A50" s="54"/>
-      <c r="B50" s="55"/>
-      <c r="C50" s="55"/>
-      <c r="D50" s="55"/>
-      <c r="E50" s="56"/>
-      <c r="F50" s="54"/>
-      <c r="G50" s="55"/>
-      <c r="H50" s="55"/>
-      <c r="I50" s="56"/>
+      <c r="A50" s="96"/>
+      <c r="B50" s="97"/>
+      <c r="C50" s="97"/>
+      <c r="D50" s="97"/>
+      <c r="E50" s="98"/>
+      <c r="F50" s="96"/>
+      <c r="G50" s="97"/>
+      <c r="H50" s="97"/>
+      <c r="I50" s="98"/>
     </row>
     <row r="51" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A51" s="60" t="s">
+      <c r="A51" s="102" t="s">
         <v>38</v>
       </c>
-      <c r="B51" s="61"/>
-      <c r="C51" s="61"/>
-      <c r="D51" s="61"/>
-      <c r="E51" s="62"/>
-      <c r="F51" s="63" t="s">
+      <c r="B51" s="103"/>
+      <c r="C51" s="103"/>
+      <c r="D51" s="103"/>
+      <c r="E51" s="104"/>
+      <c r="F51" s="105" t="s">
         <v>28</v>
       </c>
-      <c r="G51" s="64"/>
-      <c r="H51" s="64"/>
+      <c r="G51" s="106"/>
+      <c r="H51" s="106"/>
       <c r="I51" s="51" t="s">
         <v>29</v>
       </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A52" s="54" t="s">
+      <c r="A52" s="96" t="s">
         <v>30</v>
       </c>
-      <c r="B52" s="55"/>
-      <c r="C52" s="55"/>
-      <c r="D52" s="55"/>
-      <c r="E52" s="56"/>
-      <c r="F52" s="54" t="s">
+      <c r="B52" s="97"/>
+      <c r="C52" s="97"/>
+      <c r="D52" s="97"/>
+      <c r="E52" s="98"/>
+      <c r="F52" s="96" t="s">
         <v>31</v>
       </c>
-      <c r="G52" s="55"/>
-      <c r="H52" s="55"/>
+      <c r="G52" s="97"/>
+      <c r="H52" s="97"/>
       <c r="I52" s="51" t="s">
         <v>32</v>
       </c>
     </row>
     <row r="53" spans="1:9" x14ac:dyDescent="0.25">
-      <c r="A53" s="57"/>
-      <c r="B53" s="58"/>
-      <c r="C53" s="58"/>
-      <c r="D53" s="58"/>
-      <c r="E53" s="59"/>
-      <c r="F53" s="57"/>
-      <c r="G53" s="58"/>
-      <c r="H53" s="58"/>
-      <c r="I53" s="59"/>
+      <c r="A53" s="99"/>
+      <c r="B53" s="100"/>
+      <c r="C53" s="100"/>
+      <c r="D53" s="100"/>
+      <c r="E53" s="101"/>
+      <c r="F53" s="99"/>
+      <c r="G53" s="100"/>
+      <c r="H53" s="100"/>
+      <c r="I53" s="101"/>
     </row>
     <row r="54" spans="1:9" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
     <row r="55" spans="1:9" ht="21" customHeight="1" x14ac:dyDescent="0.25"/>
@@ -2930,12 +2944,51 @@
     <row r="166" ht="15" customHeight="1" x14ac:dyDescent="0.25"/>
   </sheetData>
   <mergeCells count="64">
-    <mergeCell ref="A1:D1"/>
-    <mergeCell ref="E1:I1"/>
-    <mergeCell ref="A2:D2"/>
-    <mergeCell ref="E2:I2"/>
-    <mergeCell ref="A3:D3"/>
-    <mergeCell ref="E3:I3"/>
+    <mergeCell ref="A53:E53"/>
+    <mergeCell ref="F53:I53"/>
+    <mergeCell ref="A50:E50"/>
+    <mergeCell ref="F50:I50"/>
+    <mergeCell ref="A51:E51"/>
+    <mergeCell ref="F51:H51"/>
+    <mergeCell ref="A52:E52"/>
+    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="A49:E49"/>
+    <mergeCell ref="F49:I49"/>
+    <mergeCell ref="D34:E34"/>
+    <mergeCell ref="D35:E35"/>
+    <mergeCell ref="D36:E36"/>
+    <mergeCell ref="D37:E37"/>
+    <mergeCell ref="D38:E38"/>
+    <mergeCell ref="D39:E39"/>
+    <mergeCell ref="D40:E40"/>
+    <mergeCell ref="D41:E41"/>
+    <mergeCell ref="F41:H41"/>
+    <mergeCell ref="A42:B42"/>
+    <mergeCell ref="G42:I42"/>
+    <mergeCell ref="D33:E33"/>
+    <mergeCell ref="D22:E22"/>
+    <mergeCell ref="D23:E23"/>
+    <mergeCell ref="D24:E24"/>
+    <mergeCell ref="D25:E25"/>
+    <mergeCell ref="D26:E26"/>
+    <mergeCell ref="D27:E27"/>
+    <mergeCell ref="D28:E28"/>
+    <mergeCell ref="D29:E29"/>
+    <mergeCell ref="D30:E30"/>
+    <mergeCell ref="D31:E31"/>
+    <mergeCell ref="D32:E32"/>
+    <mergeCell ref="D21:E21"/>
+    <mergeCell ref="D10:E10"/>
+    <mergeCell ref="D11:E11"/>
+    <mergeCell ref="D12:E12"/>
+    <mergeCell ref="D13:E13"/>
+    <mergeCell ref="D14:E14"/>
+    <mergeCell ref="D15:E15"/>
+    <mergeCell ref="D16:E16"/>
+    <mergeCell ref="D17:E17"/>
+    <mergeCell ref="D18:E18"/>
+    <mergeCell ref="D19:E19"/>
+    <mergeCell ref="D20:E20"/>
     <mergeCell ref="A9:G9"/>
     <mergeCell ref="H9:I9"/>
     <mergeCell ref="A4:D4"/>
@@ -2949,51 +3002,12 @@
     <mergeCell ref="B8:C8"/>
     <mergeCell ref="F8:G8"/>
     <mergeCell ref="H8:I8"/>
-    <mergeCell ref="D21:E21"/>
-    <mergeCell ref="D10:E10"/>
-    <mergeCell ref="D11:E11"/>
-    <mergeCell ref="D12:E12"/>
-    <mergeCell ref="D13:E13"/>
-    <mergeCell ref="D14:E14"/>
-    <mergeCell ref="D15:E15"/>
-    <mergeCell ref="D16:E16"/>
-    <mergeCell ref="D17:E17"/>
-    <mergeCell ref="D18:E18"/>
-    <mergeCell ref="D19:E19"/>
-    <mergeCell ref="D20:E20"/>
-    <mergeCell ref="D33:E33"/>
-    <mergeCell ref="D22:E22"/>
-    <mergeCell ref="D23:E23"/>
-    <mergeCell ref="D24:E24"/>
-    <mergeCell ref="D25:E25"/>
-    <mergeCell ref="D26:E26"/>
-    <mergeCell ref="D27:E27"/>
-    <mergeCell ref="D28:E28"/>
-    <mergeCell ref="D29:E29"/>
-    <mergeCell ref="D30:E30"/>
-    <mergeCell ref="D31:E31"/>
-    <mergeCell ref="D32:E32"/>
-    <mergeCell ref="A49:E49"/>
-    <mergeCell ref="F49:I49"/>
-    <mergeCell ref="D34:E34"/>
-    <mergeCell ref="D35:E35"/>
-    <mergeCell ref="D36:E36"/>
-    <mergeCell ref="D37:E37"/>
-    <mergeCell ref="D38:E38"/>
-    <mergeCell ref="D39:E39"/>
-    <mergeCell ref="D40:E40"/>
-    <mergeCell ref="D41:E41"/>
-    <mergeCell ref="F41:H41"/>
-    <mergeCell ref="A42:B42"/>
-    <mergeCell ref="G42:I42"/>
-    <mergeCell ref="A53:E53"/>
-    <mergeCell ref="F53:I53"/>
-    <mergeCell ref="A50:E50"/>
-    <mergeCell ref="F50:I50"/>
-    <mergeCell ref="A51:E51"/>
-    <mergeCell ref="F51:H51"/>
-    <mergeCell ref="A52:E52"/>
-    <mergeCell ref="F52:H52"/>
+    <mergeCell ref="A1:D1"/>
+    <mergeCell ref="E1:I1"/>
+    <mergeCell ref="A2:D2"/>
+    <mergeCell ref="E2:I2"/>
+    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="E3:I3"/>
   </mergeCells>
   <pageMargins left="0" right="0" top="0.47244094488188981" bottom="0" header="0" footer="0"/>
   <pageSetup paperSize="9" fitToWidth="0" orientation="portrait" r:id="rId1"/>

</xml_diff>